<commit_message>
Improve AI UI and add history chat
</commit_message>
<xml_diff>
--- a/microservices/auth_service_cus/data/cusAccList.xlsx
+++ b/microservices/auth_service_cus/data/cusAccList.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,6 +500,18 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>$2b$12$ttX6rjQxGWF2y8jXHcSWWuTWCpxxg07so7JN4MbGQYuMQQZqMDAyG</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>